<commit_message>
add oaro to treatment technologies in template
</commit_message>
<xml_diff>
--- a/backend/app/internal/assets/pareto_input_template.xlsx
+++ b/backend/app/internal/assets/pareto_input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michaelpesce/Desktop/pareto-ui/backend/app/internal/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AF01FE4-DBFA-B94C-B276-A208E601EED8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D9F1CA-2B51-334E-B94C-E4913AE45CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12340" yWindow="760" windowWidth="21560" windowHeight="18900" tabRatio="953" xr2:uid="{FB8C51AB-905F-4544-9E4B-1F4384FA855C}"/>
   </bookViews>
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="306">
   <si>
     <t>Data Input Spreadsheet Overview</t>
   </si>
@@ -3242,7 +3242,9 @@
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A6" s="5"/>
+      <c r="A6" s="2" t="s">
+        <v>274</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:A5" xr:uid="{2C820352-28DB-4692-BCE8-9A9846CC4956}"/>

</xml_diff>

<commit_message>
fix references in excel template
</commit_message>
<xml_diff>
--- a/backend/app/internal/assets/pareto_input_template.xlsx
+++ b/backend/app/internal/assets/pareto_input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michaelpesce/Desktop/pareto-ui/backend/app/internal/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81D9F1CA-2B51-334E-B94C-E4913AE45CBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF34D6B0-AA3A-E44A-99C3-26716B4DA864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12340" yWindow="760" windowWidth="21560" windowHeight="18900" tabRatio="953" xr2:uid="{FB8C51AB-905F-4544-9E4B-1F4384FA855C}"/>
+    <workbookView xWindow="16760" yWindow="760" windowWidth="17800" windowHeight="19320" tabRatio="953" xr2:uid="{FB8C51AB-905F-4544-9E4B-1F4384FA855C}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="33" r:id="rId1"/>
@@ -107,9 +107,9 @@
     <sheet name="ExternalWaterQuality" sheetId="147" r:id="rId92"/>
     <sheet name="PadWaterQuality" sheetId="99" r:id="rId93"/>
     <sheet name="StorageInitialWaterQuality" sheetId="100" r:id="rId94"/>
-    <sheet name="PadStorageInitialWaterQuality" sheetId="101" r:id="rId95"/>
-    <sheet name="AirEmissionCoefficients" sheetId="145" r:id="rId96"/>
-    <sheet name="TreatmentEmissionCoefficients" sheetId="144" r:id="rId97"/>
+    <sheet name="AirEmissionCoefficients" sheetId="145" r:id="rId95"/>
+    <sheet name="TreatmentEmissionCoefficients" sheetId="144" r:id="rId96"/>
+    <sheet name="PadStorageInitialWaterQuality" sheetId="101" r:id="rId97"/>
     <sheet name="TreatmentExpansionLeadTime" sheetId="128" r:id="rId98"/>
     <sheet name="DisposalExpansionLeadTime" sheetId="129" r:id="rId99"/>
     <sheet name="StorageExpansionLeadTime" sheetId="130" r:id="rId100"/>
@@ -2659,9 +2659,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Storage Expansion Lead Time [",VLOOKUP("decision period",#REF!, 2, FALSE),"s]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Storage Expansion Lead Time [",VLOOKUP("decision period", Units!$A$2:$B$11, 2, FALSE),"s]")</f>
+        <v>Table of Storage Expansion Lead Time [weeks]</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2713,9 +2713,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Pipeline Expansion Lead Time - Distance Based [",VLOOKUP("decision period",#REF!, 2, FALSE),"s/",VLOOKUP("distance",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Pipeline Expansion Lead Time - Distance Based [",VLOOKUP("decision period", Units!$A$2:$B$11, 2, FALSE),"s/",VLOOKUP("distance", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Pipeline Expansion Lead Time - Distance Based [weeks/mile]</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
@@ -5743,9 +5743,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:55" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Completions Water Demand for Completions Sites over ",VLOOKUP("decision period",#REF!, 2, FALSE),"s [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Completions Water Demand for Completions Sites over ",VLOOKUP("decision period", Units!$A$2:$B$11, 2, FALSE),"s [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Completions Water Demand for Completions Sites over weeks [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:55" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -6044,9 +6044,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Production Rate Forecasts by Pads [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Production Rate Forecasts by Pads [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Production Rate Forecasts by Pads [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:53" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -6464,9 +6464,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Flowback Rate Forecasts by Pads [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Flowback Rate Forecasts by Pads [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Flowback Rate Forecasts by Pads [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:53" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -7875,9 +7875,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Initial Pipeline Capacity between Sites [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Initial Pipeline Capacity between Sites [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Initial Pipeline Capacity between Sites [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -12403,9 +12403,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Initial Disposal Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Initial Disposal Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Initial Disposal Capacity [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -12443,9 +12443,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Initial Storage Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Initial Storage Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Initial Storage Capacity [bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -12487,9 +12487,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Initial Treatment Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Initial Treatment Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Initial Treatment Capacity [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -12537,9 +12537,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Beneficial Reuse minimum required flow [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Beneficial Reuse minimum required flow [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Beneficial Reuse minimum required flow [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
@@ -12886,9 +12886,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Beneficial Reuse Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"] (leave cells blank to indicate infinite capacity)")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Beneficial Reuse Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"] (leave cells blank to indicate infinite capacity)")</f>
+        <v>Table of Beneficial Reuse Capacity [bbl/day] (leave cells blank to indicate infinite capacity)</v>
       </c>
     </row>
     <row r="2" spans="1:53" x14ac:dyDescent="0.2">
@@ -13278,9 +13278,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:53" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of External Water Sourcing Availability [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of External Water Sourcing Availability [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of External Water Sourcing Availability [bbl/day]</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>105</v>
@@ -13596,9 +13596,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Completions Pad Storage Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Completions Pad Storage Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Completions Pad Storage Capacity [bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -13632,9 +13632,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Pad Offloading Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Pad Offloading Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Pad Offloading Capacity [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -13669,9 +13669,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Node Capacity Capacity [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]", " *absence of node or empty cell signifies no max capacity")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Node Capacity Capacity [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]", " *absence of node or empty cell signifies no max capacity")</f>
+        <v>Table of Node Capacity Capacity [bbl/day] *absence of node or empty cell signifies no max capacity</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -13943,9 +13943,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Disposal Operational Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Disposal Operational Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Disposal Operational Cost [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -13983,9 +13983,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Treatment Operational Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Treatment Operational Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Treatment Operational Cost [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
@@ -14068,9 +14068,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Reuse Operational Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Reuse Operational Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Reuse Operational Cost [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -14104,9 +14104,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Pipeline Operational Cost between Sites [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Pipeline Operational Cost between Sites [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Pipeline Operational Cost between Sites [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -14637,9 +14637,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of External Water Souring Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of External Water Souring Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of External Water Souring Cost [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -14718,9 +14718,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Trucking Hourly Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/", "hour","]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Trucking Hourly Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", "hour","]")</f>
+        <v>Table of Trucking Hourly Cost [USD/hour]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -14833,9 +14833,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Disposal Capacity Expansion Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/(", VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),")]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Disposal Capacity Expansion Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/(", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),")]")</f>
+        <v>Table of Disposal Capacity Expansion Cost [USD/(bbl/day)]</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -14881,9 +14881,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Disposal Capacity Expansion Increments [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Disposal Capacity Expansion Increments [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Disposal Capacity Expansion Increments [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -14929,9 +14929,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Storage Capacity Expansion Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Storage Capacity Expansion Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Storage Capacity Expansion Cost [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -14983,9 +14983,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Storage Capacity Expansion Increments [",VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Storage Capacity Expansion Increments [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Storage Capacity Expansion Increments [bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -15032,9 +15032,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Treatment Capacity Expansion Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/(", VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),")]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Treatment Capacity Expansion Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/(", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),")]")</f>
+        <v>Table of Treatment Capacity Expansion Cost [USD/(bbl/day)]</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -15150,9 +15150,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Treatment Capacity Expansion Increments [",VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Treatment Capacity Expansion Increments [",VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Treatment Capacity Expansion Increments [bbl/day]</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
@@ -15225,9 +15225,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Pipeline Expansion Cost [",VLOOKUP("currency",#REF!, 2, FALSE),"/(", VLOOKUP("diameter",#REF!, 2, FALSE),"-", VLOOKUP("distance",#REF!, 2, FALSE),")]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Pipeline Expansion Cost [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/(", VLOOKUP("diameter", Units!$A$2:$B$11, 2, FALSE),"-", VLOOKUP("distance", Units!$A$2:$B$11, 2, FALSE),")]")</f>
+        <v>Pipeline Expansion Cost [USD/(inch-mile)]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -15263,9 +15263,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Pipeline Expansion Distances [",VLOOKUP("distance",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Pipeline Expansion Distances [",VLOOKUP("distance", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Pipeline Expansion Distances [mile]</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
@@ -15833,9 +15833,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Pipeline Capacity Expansion Costs [",VLOOKUP("currency",#REF!, 2, FALSE),"/(", VLOOKUP("volume",#REF!, 2, FALSE),"/", VLOOKUP("time",#REF!, 2, FALSE),")]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Pipeline Capacity Expansion Costs [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/(", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("time", Units!$A$2:$B$11, 2, FALSE),")]")</f>
+        <v>Table of Pipeline Capacity Expansion Costs [USD/(bbl/day)]</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -15960,9 +15960,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Pipeline Diameters [",VLOOKUP("diameter",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Pipeline Diameters [",VLOOKUP("diameter", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Pipeline Diameters [inch]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -16297,9 +16297,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table with credit received for sending water to beneficial reuse [",VLOOKUP("currency",#REF!, 2, FALSE),"/", VLOOKUP("volume",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table with credit received for sending water to beneficial reuse [",VLOOKUP("currency", Units!$A$2:$B$11, 2, FALSE),"/", VLOOKUP("volume", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table with credit received for sending water to beneficial reuse [USD/bbl]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -16562,9 +16562,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Water Quality of Produced Water and Flowback Water [",VLOOKUP("concentration",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Water Quality of Produced Water and Flowback Water [",VLOOKUP("concentration", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Water Quality of Produced Water and Flowback Water [mg/liter]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -16615,9 +16615,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Initial Water Quality at Storage [", VLOOKUP("concentration",#REF!, 2, FALSE),,"]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Initial Water Quality at Storage [", VLOOKUP("concentration", Units!A2:B9, 2, FALSE),,"]")</f>
+        <v>Table of Initial Water Quality at Storage [mg/liter]</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -16648,42 +16648,6 @@
 </file>
 
 <file path=xl/worksheets/sheet95.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA334136-9628-4654-B8E2-BCFE701B0D1B}">
-  <sheetPr>
-    <tabColor theme="8" tint="0.79998168889431442"/>
-  </sheetPr>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="17.6640625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="9.1640625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Initial Water Quality at Completions Pad Storage [",VLOOKUP("concentration",#REF!, 2, FALSE),"]")</f>
-        <v>#REF!</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="58"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet96.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73C69F2D-49DC-1944-BFFB-2EEA9F71D13F}">
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
@@ -16832,7 +16796,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet97.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet96.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE0936AA-9CB5-FA48-AA26-19FC94AF5C3A}">
   <sheetPr>
     <tabColor theme="8" tint="0.79998168889431442"/>
@@ -16973,6 +16937,42 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet97.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AA334136-9628-4654-B8E2-BCFE701B0D1B}">
+  <sheetPr>
+    <tabColor theme="8" tint="0.79998168889431442"/>
+  </sheetPr>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="9.1640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Initial Water Quality at Completions Pad Storage [",VLOOKUP("concentration", Units!$A$2:$B$11, 2, FALSE),"]")</f>
+        <v>Table of Initial Water Quality at Completions Pad Storage [mg/liter]</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="6"/>
+      <c r="B3" s="58"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -16989,9 +16989,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Treatment Expansion Lead Time [",VLOOKUP("decision period",#REF!, 2, FALSE),"s]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Treatment Expansion Lead Time [",VLOOKUP("decision period", Units!$A$2:$B$11, 2, FALSE),"s]")</f>
+        <v>Table of Treatment Expansion Lead Time [weeks]</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -17113,9 +17113,9 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="e">
-        <f>_xlfn.CONCAT( "Table of Disposal Expansion Lead Time [",VLOOKUP("decision period",#REF!, 2, FALSE),"s]")</f>
-        <v>#REF!</v>
+      <c r="A1" s="1" t="str">
+        <f>_xlfn.CONCAT( "Table of Disposal Expansion Lead Time [",VLOOKUP("decision period", Units!$A$2:$B$11, 2, FALSE),"s]")</f>
+        <v>Table of Disposal Expansion Lead Time [weeks]</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>

</xml_diff>

<commit_message>
add headers to missing R arc tabs
</commit_message>
<xml_diff>
--- a/backend/app/internal/assets/pareto_input_template.xlsx
+++ b/backend/app/internal/assets/pareto_input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michaelpesce/Desktop/pareto-ui/backend/app/internal/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF34D6B0-AA3A-E44A-99C3-26716B4DA864}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0343C21-CC0E-CE4A-8B38-676F0769AC96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="16760" yWindow="760" windowWidth="17800" windowHeight="19320" tabRatio="953" xr2:uid="{FB8C51AB-905F-4544-9E4B-1F4384FA855C}"/>
   </bookViews>
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="846" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="848" uniqueCount="306">
   <si>
     <t>Data Input Spreadsheet Overview</t>
   </si>
@@ -5097,15 +5097,21 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="9.1640625" style="1"/>
+    <col min="1" max="1" width="15.33203125" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>259</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -5592,15 +5598,21 @@
   <sheetPr>
     <tabColor theme="9" tint="0.79998168889431442"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="16384" width="9.1640625" style="1"/>
+    <col min="1" max="1" width="15.6640625" style="1" customWidth="1"/>
+    <col min="2" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>260</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>